<commit_message>
style(site): relecture complète des textes, en anglais et en français
Toutes les pages réécrites dans une langue plus directe : phrases plus
courtes, moins de formules, première personne là où c'est une personne
qui parle (contact, page A-123). Titres simplifiés, intitulés de
l'offre alignés (« Toolkits, Training & Software »). La checklist PDF
et le classeur gratuit sont régénérés avec les mêmes corrections.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/A-123-2026-Quick-Check.xlsx
+++ b/downloads/A-123-2026-Quick-Check.xlsx
@@ -27,7 +27,7 @@
     <t>Grey cells</t>
   </si>
   <si>
-    <t>Formulas — leave them.</t>
+    <t>Formulas. Leave them alone.</t>
   </si>
   <si>
     <t>Italic grey rows</t>
@@ -159,7 +159,7 @@
     <t>R-001</t>
   </si>
   <si>
-    <t>Grants management — discretionary awards</t>
+    <t>Grants management, discretionary awards</t>
   </si>
   <si>
     <t>Payments to recipients are accurate, allowable, and supported (2 CFR 200).</t>
@@ -327,7 +327,7 @@
     <t>Not yet answered:</t>
   </si>
   <si>
-    <t>Under the 2026 circular, non-achievement of a relevant principle results in a material weakness (Table 2). A "No" here is not yet a conclusion — it is the place to start.</t>
+    <t>Under the 2026 circular, non-achievement of a relevant principle results in a material weakness (Table 2). A "No" here is not yet a conclusion, it is the place to start.</t>
   </si>
   <si>
     <t>Month</t>

</xml_diff>